<commit_message>
update 17 feb 2023
</commit_message>
<xml_diff>
--- a/Kas Hima - yrw - stthf.xlsx
+++ b/Kas Hima - yrw - stthf.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/03461a0c230c1ba6/Documents/Yofandi/rekap data - uang galon^J parkir^J bumbu asrama/uanghimastthf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{B3173F7A-21FF-40BD-9CB1-EB632A60ABC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85B6E048-349F-43F1-841A-FE5E31CA27F8}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{B3173F7A-21FF-40BD-9CB1-EB632A60ABC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{112807E6-186B-4796-BCCA-D74F46D990B4}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="21792" windowHeight="12120" xr2:uid="{B1E7B7C2-6564-4E00-949B-823A851BA38E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>*dimulai tanggal 14 Maret 2022</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>uang persembahan - reguler - valentine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cynta </t>
+  </si>
+  <si>
+    <t>yofandi</t>
   </si>
 </sst>
 </file>
@@ -88,7 +94,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,13 +108,33 @@
       <name val="Agency FB"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -120,18 +146,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="60% - Accent1" xfId="1" builtinId="32"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -460,38 +490,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -504,22 +534,22 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -540,6 +570,9 @@
       <c r="E9" t="s">
         <v>9</v>
       </c>
+      <c r="F9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
@@ -558,6 +591,9 @@
       <c r="E10" t="s">
         <v>10</v>
       </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
@@ -576,6 +612,9 @@
       <c r="E11" t="s">
         <v>11</v>
       </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
@@ -594,6 +633,9 @@
       <c r="E12" t="s">
         <v>10</v>
       </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
@@ -612,6 +654,9 @@
       <c r="E13" t="s">
         <v>12</v>
       </c>
+      <c r="F13" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
@@ -621,14 +666,17 @@
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <v>436000</v>
+        <v>361500</v>
       </c>
       <c r="D14" s="2">
         <f t="shared" si="0"/>
-        <v>67100</v>
+        <v>141600</v>
       </c>
       <c r="E14" t="s">
         <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -643,18 +691,34 @@
       </c>
       <c r="D15" s="2">
         <f t="shared" si="0"/>
-        <v>162600</v>
+        <v>237100</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
       </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="A16" s="1">
+        <v>44974</v>
+      </c>
+      <c r="B16" s="2">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>7500</v>
+      </c>
       <c r="D16" s="2">
         <f t="shared" si="0"/>
-        <v>162600</v>
+        <v>229600</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
@@ -662,7 +726,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="2">
         <f t="shared" si="0"/>
-        <v>162600</v>
+        <v>229600</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
update 01 Mar 2023
</commit_message>
<xml_diff>
--- a/Kas Hima - yrw - stthf.xlsx
+++ b/Kas Hima - yrw - stthf.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/03461a0c230c1ba6/Documents/Yofandi/rekap data - uang galon^J parkir^J bumbu asrama/uanghimastthf/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yofan\OneDrive\Documents\Yofandi\rekap data - uang galon, parkir, bumbu asrama\uanghimastthf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{B3173F7A-21FF-40BD-9CB1-EB632A60ABC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{112807E6-186B-4796-BCCA-D74F46D990B4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EE9A89-DFF8-43B5-8828-2C097721B8F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="768" yWindow="768" windowWidth="21792" windowHeight="12120" xr2:uid="{B1E7B7C2-6564-4E00-949B-823A851BA38E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
   <si>
     <t>*dimulai tanggal 14 Maret 2022</t>
   </si>
@@ -175,10 +175,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -721,42 +717,55 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>44986</v>
+      </c>
+      <c r="B17" s="2">
+        <v>110200</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0</v>
+      </c>
       <c r="D17" s="2">
         <f t="shared" si="0"/>
-        <v>229600</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+        <v>339800</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D27" s="2"/>
     </row>
   </sheetData>

</xml_diff>